<commit_message>
perf: serve chapter puzzles as optimized webp
</commit_message>
<xml_diff>
--- a/references/annual-bank-template/questions.xlsx
+++ b/references/annual-bank-template/questions.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="questions" sheetId="1" r:id="R77e2036083c44038"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="questions" sheetId="1" r:id="R8875fbb474e0478b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -471,7 +471,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F2" s="29" t="str">
-        <x:v>chapter-01.png</x:v>
+        <x:v>chapter-01.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -489,7 +489,7 @@
         <x:v>number</x:v>
       </x:c>
       <x:c r="F3" s="29" t="str">
-        <x:v>chapter-02.png</x:v>
+        <x:v>chapter-02.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -507,7 +507,7 @@
         <x:v>zh</x:v>
       </x:c>
       <x:c r="F4" s="29" t="str">
-        <x:v>chapter-03.png</x:v>
+        <x:v>chapter-03.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -525,7 +525,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F5" s="29" t="str">
-        <x:v>chapter-04.png</x:v>
+        <x:v>chapter-04.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -543,7 +543,7 @@
         <x:v>number</x:v>
       </x:c>
       <x:c r="F6" s="29" t="str">
-        <x:v>chapter-05.png</x:v>
+        <x:v>chapter-05.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -561,7 +561,7 @@
         <x:v>zh</x:v>
       </x:c>
       <x:c r="F7" s="29" t="str">
-        <x:v>chapter-06.png</x:v>
+        <x:v>chapter-06.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -579,7 +579,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F8" s="29" t="str">
-        <x:v>chapter-07.png</x:v>
+        <x:v>chapter-07.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -597,7 +597,7 @@
         <x:v>zh</x:v>
       </x:c>
       <x:c r="F9" s="29" t="str">
-        <x:v>chapter-08.png</x:v>
+        <x:v>chapter-08.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -615,7 +615,7 @@
         <x:v>number</x:v>
       </x:c>
       <x:c r="F10" s="29" t="str">
-        <x:v>chapter-09.png</x:v>
+        <x:v>chapter-09.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -633,7 +633,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F11" s="29" t="str">
-        <x:v>chapter-10.png</x:v>
+        <x:v>chapter-10.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -651,7 +651,7 @@
         <x:v>zh</x:v>
       </x:c>
       <x:c r="F12" s="29" t="str">
-        <x:v>chapter-11.png</x:v>
+        <x:v>chapter-11.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -669,7 +669,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F13" s="29" t="str">
-        <x:v>chapter-12.png</x:v>
+        <x:v>chapter-12.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -687,7 +687,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F14" s="29" t="str">
-        <x:v>chapter-13.png</x:v>
+        <x:v>chapter-13.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -705,7 +705,7 @@
         <x:v>zh</x:v>
       </x:c>
       <x:c r="F15" s="29" t="str">
-        <x:v>chapter-14.png</x:v>
+        <x:v>chapter-14.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -723,7 +723,7 @@
         <x:v>zh</x:v>
       </x:c>
       <x:c r="F16" s="29" t="str">
-        <x:v>chapter-15.png</x:v>
+        <x:v>chapter-15.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -741,7 +741,7 @@
         <x:v>number</x:v>
       </x:c>
       <x:c r="F17" s="29" t="str">
-        <x:v>chapter-16.png</x:v>
+        <x:v>chapter-16.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -759,7 +759,7 @@
         <x:v>zh</x:v>
       </x:c>
       <x:c r="F18" s="29" t="str">
-        <x:v>chapter-17.png</x:v>
+        <x:v>chapter-17.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -777,7 +777,7 @@
         <x:v>number</x:v>
       </x:c>
       <x:c r="F19" s="29" t="str">
-        <x:v>chapter-18.png</x:v>
+        <x:v>chapter-18.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -795,7 +795,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F20" s="29" t="str">
-        <x:v>chapter-19.png</x:v>
+        <x:v>chapter-19.webp</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -813,7 +813,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F21" s="33" t="str">
-        <x:v>chapter-20.png</x:v>
+        <x:v>chapter-20.webp</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>